<commit_message>
tracker: confirm Sir Tristan free-departure (NEFE5L) — row 30 ? -> Y
The power has no dedicated log line (only a client toast), but its effect is
provable: Turn 6 Chrome moved from the Round Table to Excalibur (7:34:26) and
took a second heroic action (move Excalibur, 7:34:31) with no "sacrificed 1 LP"
line between them — only Tristan's free departure permits a RT departure plus a
second action without a sacrifice. Recurs Turn 15 (Saxon War) and Turn 18 (Holy
Grail).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Game_Coverage_Tracker.xlsx
+++ b/Game_Coverage_Tracker.xlsx
@@ -1271,7 +1271,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
@@ -2323,7 +2322,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2343,7 +2342,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>in play (Tristan); free-departure not separately logged</t>
+          <t>Free departure: no separate log line (client toast only); provable via move-from-RT + 2nd heroic action with no sacrifice. Turn 6 (to Excalibur), Turn 15 (to Saxon War), Turn 18 (to Holy Grail).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix 12th-sword Traitor reveal/flip skipped on non-host trigger (v97)
checkGameEnd() gated the endgame Traitor reveal + 2 White->Black flip behind isHost, but it runs on the client that placed the 12th sword. A non-host trigger (e.g. a player completing the war that places the 12th sword) skipped the flip and scored the unflipped board, recording a Traitor win as a loyal win (HMXQCW: 7W-5B loyal instead of Evil). Extracted finalizeSwordCountEnd() and delegate the tally to the host via a new finalizeSwordCount drawRequest (mirrors accuseReveal/writeLoyalties). Bump v96->v97; record HMXQCW in coverage tracker.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Game_Coverage_Tracker.xlsx
+++ b/Game_Coverage_Tracker.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="21.33203125" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -910,6 +910,43 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>t45 traitor-taunt stall (fixed v94); revealed traitor wrongly received Lancelot Armor (fixed v95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HMXQCW</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>6/14/2026 8:00 AM - 6/15 10:35 PM</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>v96</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Arthur=iPhone Chrome (TRAITOR); Galahad=Picky Safari; Kay=iPhone Firefox; host=Edge PC spectator</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Loyal "win" 7W-5B - INCORRECT: Traitor (Arthur) unrevealed; 12th-sword reveal/flip bug</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BUG: non-host 12th-sword Traitor reveal/flip skipped (fixed v97). Locked host PC -&gt; heartbeat-stale churn/lag (op). Benign IndexedDB auth-persistence log noise t19-30 (no gameplay impact).</t>
         </is>
       </c>
     </row>
@@ -993,7 +1030,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>XF4V2C (6/13)</t>
+          <t>XF4V2C (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -1003,7 +1040,7 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>VJCEXL (6/8); KLF2RQ x2 (6/11); HXZ4HU (6/12); F2EXND (6/13); NEFE5L (6/13)</t>
+          <t>VJCEXL (6/8); KLF2RQ x2 (6/11); HXZ4HU (6/12); F2EXND (6/13); NEFE5L (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
@@ -1030,7 +1067,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>VJCEXL (6/8); KLF2RQ (6/11); XF4V2C (6/13); F2EXND (6/13); NEFE5L (6/13)</t>
+          <t>VJCEXL (6/8); KLF2RQ (6/11); XF4V2C (6/13); F2EXND (6/13); NEFE5L (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -1072,17 +1109,17 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>LOSS NOT YET OBSERVED -- only active after Lancelot ends; not reached in XF4V2C/F2EXND</t>
+          <t>First loss observed HMXQCW (6/15): 5th Dragon card forced combat, no knight present -&gt; 2 Black Swords, -2 LP</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1151,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>F2EXND (6/13)</t>
+          <t>F2EXND (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1141,7 +1178,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>VJCEXL (6/8); KLF2RQ (6/11); HXZ4HU (6/12); NEFE5L (6/13)</t>
+          <t>VJCEXL (6/8); KLF2RQ (6/11); HXZ4HU (6/12); NEFE5L (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1215,7 +1252,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>XF4V2C (6/13); F2EXND (6/13)</t>
+          <t>XF4V2C (6/13); F2EXND (6/13); HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1279,7 +1316,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dragon's Quest LOST | Siege Engine fight LOST</t>
+          <t>Siege Engine fight LOST</t>
         </is>
       </c>
     </row>
@@ -1465,6 +1502,11 @@
           <t>Evil win - black majority at 12 swords</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Would have been HMXQCW (6/15): 7W -&gt; flip 2 -&gt; 5W/7B (black majority + 7 black = Evil), but v96 non-host flip bug recorded a loyal win; re-test after v97 fix</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1923,7 +1965,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>accused in both completed games so far</t>
+          <t>HMXQCW (6/15) reached the 12th sword with the Traitor (Arthur) still hidden, but the v96 non-host bug skipped the reveal/flip; re-test after the v97 fix</t>
         </is>
       </c>
     </row>
@@ -1973,6 +2015,31 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>False accusation (penalty)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>HMXQCW</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>6/15/2026</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>v96</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Arthur-&gt;Galahad (t16) &amp; Galahad-&gt;Kay (t17), both Loyal; penalty no-op (0 swords on table at the time)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: record HMXQCW siege-fight loss (closes last 'not yet observed' gap)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Game_Coverage_Tracker.xlsx
+++ b/Game_Coverage_Tracker.xlsx
@@ -1294,17 +1294,17 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>HMXQCW (6/15)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>SUPPLEMENTARY -- a siege-fight LOSS (sum &lt;= d8 -&gt; lose 1 LP, engine stays) NOT YET OBSERVED</t>
+          <t>SUPPLEMENTARY -- siege-fight LOSS first observed HMXQCW (6/15): Kay Fight 3 vs d8=5 -&gt; lost 1 LP, engine stayed (t9). Many wins across all games.</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Siege Engine fight LOST</t>
+          <t>none -- all observed as of HMXQCW (6/15)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: record TP3TFA (v99 spectator-host game, Evil win 12 siege)
First clean spectator-host game on v99 (forgot-"Spectator" fix validated).
- Games: add TP3TFA (28 turns, Evil win via 12 Siege Engines, traitor
  Percival self-revealed via Fate t12).
- Quest Outcomes: Black Knight / Lancelot / Excalibur won; Holy Grail lost
  (standard fill-loss: 5 Despair + 1 Desolation -> 3 Black Swords, t10).
- Coverage: append TP3TFA across 30 demonstrated rows.
- Logged two deferred future improvements in the game's Notable Issues:
  spectator-host Merlin auto-pass (log noise); cinematic autoplay-stall on
  a backgrounded tab. No code change / no version bump.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Game_Coverage_Tracker.xlsx
+++ b/Game_Coverage_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Games" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Quest Outcomes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Games" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest Outcomes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Games'!$A$1:$G$7</definedName>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="21.33203125" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -947,6 +947,41 @@
       <c r="G12" t="inlineStr">
         <is>
           <t>BUG: non-host 12th-sword Traitor reveal/flip skipped (fixed v97). Locked host PC -&gt; heartbeat-stale churn/lag (op). Benign IndexedDB auth-persistence log noise t19-30 (no gameplay impact).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TP3TFA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>6/25/2026 7:58-8:17 PM</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>v99</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Picky Safari = King Arthur; iPhone Firefox = Sir Galahad; iPhone Google Chrome = Sir Percival (TRAITOR); host = Edge PC spectator</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>28</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Evil win - 12 Siege Engines surround Camelot (traitor Percival self-revealed via Fate t12)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>First clean spectator-host game on v99 (forgot-"Spectator" fix validated; game completed). FUTURE IMPROVEMENTS (deferred): (1) spectator host auto-passes Merlin votes via _spectator quarantine - log noise, inert (renderMerlinCancelPanel); (2) Excalibur-win cinematic stalled on backgrounded Firefox tab (autoplay blocked while driving 3 players on one phone), needed manual Skip - harden onCinematicChanged to auto-dismiss when playback cannot start.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1065,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>XF4V2C (6/13); HMXQCW (6/15)</t>
+          <t>XF4V2C (6/13); HMXQCW (6/15); TP3TFA (6/25)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -1067,7 +1102,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>VJCEXL (6/8); KLF2RQ (6/11); XF4V2C (6/13); F2EXND (6/13); NEFE5L (6/13); HMXQCW (6/15)</t>
+          <t>VJCEXL (6/8); KLF2RQ (6/11); XF4V2C (6/13); F2EXND (6/13); NEFE5L (6/13); HMXQCW (6/15); TP3TFA (6/25)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -1141,7 +1176,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>VJCEXL (6/8); KLF2RQ (6/11); HXZ4HU (6/12); NEFE5L (6/13)</t>
+          <t>VJCEXL (6/8); KLF2RQ (6/11); HXZ4HU (6/12); NEFE5L (6/13); TP3TFA (6/25)</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1188,12 +1223,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>F2EXND (6/13)</t>
+          <t>F2EXND (6/13); TP3TFA (6/25)</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Loss (F2EXND) = 7 black on board + Desolation; pushed Round Table to 7+ Black Swords -&gt; game over</t>
+          <t>Loss (F2EXND) = 7 black on board + Desolation; pushed Round Table to 7+ Black Swords -&gt; game over | TP3TFA (6/25): standard fill-loss - 5 Despair + 1 Desolation -&gt; 3 Black Swords, Grail removed (t10)</t>
         </is>
       </c>
     </row>
@@ -1472,22 +1507,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>XF4V2C; NEFE5L</t>
+          <t>XF4V2C; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6/13/2026; 6/13/2026</t>
+          <t>6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>v91; v93</t>
+          <t>v91; v93; v99</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>GAME OVER: 12 Siege Engines surround Camelot (t38); traitor Arthur added the 11th, Kay forced the 12th</t>
+          <t>GAME OVER: 12 Siege Engines surround Camelot (t38); traitor Arthur added the 11th, Kay forced the 12th | TP3TFA: traitor Percival added several; Arthur forced the 12th (t28)</t>
         </is>
       </c>
     </row>
@@ -1600,22 +1635,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v93</t>
+          <t>v7x; v84; v87; v93; v99</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>relic to Chrome (6/8) / Arthur-Firefox +Heroism extra sword (6/11) | HXZ4HU: relic to Gawain/Firefox</t>
+          <t>relic to Chrome (6/8) / Arthur-Firefox +Heroism extra sword (6/11) | HXZ4HU: relic to Gawain/Firefox | TP3TFA: relic to Galahad/Firefox (t11)</t>
         </is>
       </c>
     </row>
@@ -1637,22 +1672,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KLF2RQ; HXZ4HU</t>
+          <t>KLF2RQ; HXZ4HU; TP3TFA</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>6/12/2026; 6/12/2026</t>
+          <t>6/12/2026; 6/12/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>v84; v87</t>
+          <t>v84; v87; v99</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>narrative log line added in v87 ('Excalibur (holder) adds +1 to the combat total: X -&gt; Y') - provable from next game; KLF2RQ siege Fight-9 wins were fight cards, passive applies to quest combat only | HXZ4HU: 'Excalibur (Firefox) adds +1: 36-&gt;37' on Dragon win</t>
+          <t>narrative log line added in v87 ('Excalibur (holder) adds +1 to the combat total: X -&gt; Y') - provable from next game; KLF2RQ siege Fight-9 wins were fight cards, passive applies to quest combat only | HXZ4HU: 'Excalibur (Firefox) adds +1: 36-&gt;37' on Dragon win | TP3TFA: 'Excalibur (Firefox) adds +1: 10-&gt;11' on Black Knight win (t23)</t>
         </is>
       </c>
     </row>
@@ -1822,22 +1857,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>v7x; v84; v91; v92; v93</t>
+          <t>v7x; v84; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lancelot quest won both games | XF4V2C: Kay won Lancelot t21 | F2EXND: Palamedes won Lancelot t22</t>
+          <t>Lancelot quest won both games | XF4V2C: Kay won Lancelot t21 | F2EXND: Palamedes won Lancelot t22 | TP3TFA: Arthur won Lancelot (t25)</t>
         </is>
       </c>
     </row>
@@ -2061,22 +2096,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>HXZ4HU; XF4V2C</t>
+          <t>HXZ4HU; XF4V2C; TP3TFA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>6/12/2026; 6/13/2026</t>
+          <t>6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>v87; v91</t>
+          <t>v87; v91; v99</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Chrome/Tristan played Fate -&gt; revealed himself (t37) | XF4V2C: Arthur played Fate -&gt; revealed t37</t>
+          <t>Chrome/Tristan played Fate -&gt; revealed himself (t37) | XF4V2C: Arthur played Fate -&gt; revealed t37 | TP3TFA: Percival/Chrome played Fate -&gt; revealed (t12)</t>
         </is>
       </c>
     </row>
@@ -2098,22 +2133,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>VJCEXL; HXZ4HU; NEFE5L</t>
+          <t>VJCEXL; HXZ4HU; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>6/9/2026; 6/12/2026; 6/13/2026</t>
+          <t>6/9/2026; 6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>v76; v87; v93</t>
+          <t>v76; v87; v93; v99</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>"Traitor stole a card from iPhone Google Chrome!" | HXZ4HU: multiple taunts (Firefox &amp; Safari)</t>
+          <t>"Traitor stole a card from iPhone Google Chrome!" | HXZ4HU: multiple taunts (Firefox &amp; Safari) | TP3TFA: stole from Arthur/Galahad ~6x (t12-t27)</t>
         </is>
       </c>
     </row>
@@ -2172,22 +2207,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; TP3TFA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92</t>
+          <t>v7x; v84; v87; v91; v92; v99</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>~12 exchanges in KLF2RQ | HXZ4HU: ~10 exchanges | XF4V2C: several exchanges | F2EXND: several exchanges</t>
+          <t>~12 exchanges in KLF2RQ | HXZ4HU: ~10 exchanges | XF4V2C: several exchanges | F2EXND: several exchanges | TP3TFA: exchanges t4/t7/t10</t>
         </is>
       </c>
     </row>
@@ -2209,22 +2244,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ</t>
+          <t>VJCEXL; KLF2RQ; TP3TFA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>v7x; v84</t>
+          <t>v7x; v84; v99</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>~12 free plays in KLF2RQ (8 different cards)</t>
+          <t>~12 free plays in KLF2RQ (8 different cards) | TP3TFA: Reinforcements t5, Lady of the Lake t8, Merlin t23</t>
         </is>
       </c>
     </row>
@@ -2357,22 +2392,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NEFE5L</t>
+          <t>NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>6/13/2026</t>
+          <t>6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>v93</t>
+          <t>v93; v99</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>narrative log line added in v87 ('peeked at the top Black card') - in play both completed games but unlogged until now | NEFE5L: peeked ~18x (provable)</t>
+          <t>narrative log line added in v87 ('peeked at the top Black card') - in play both completed games but unlogged until now | NEFE5L: peeked ~18x (provable) | TP3TFA: peeked t3/t6/t9/t12</t>
         </is>
       </c>
     </row>
@@ -2503,22 +2538,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>KLF2RQ; HXZ4HU; XF4V2C; NEFE5L</t>
+          <t>KLF2RQ; HXZ4HU; XF4V2C; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>v84; v87; v91; v93</t>
+          <t>v84; v87; v91; v93; v99</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2 uses | HXZ4HU: several uses | XF4V2C: Chrome t22</t>
+          <t>2 uses | HXZ4HU: several uses | XF4V2C: Chrome t22 | TP3TFA: Galahad removed 1 siege (t23)</t>
         </is>
       </c>
     </row>
@@ -2614,22 +2649,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v92; v93</t>
+          <t>v7x; v84; v87; v92; v93; v99</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>HXZ4HU: t36 | F2EXND: Kay t12 | NEFE5L: each-knight-draws-1 variant</t>
+          <t>HXZ4HU: t36 | F2EXND: Kay t12 | NEFE5L: each-knight-draws-1 variant | TP3TFA: Galahad drew 4 (t5)</t>
         </is>
       </c>
     </row>
@@ -2725,22 +2760,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>6/9/2026; 6/11/2026; 6/12/2026; 6/13/2026</t>
+          <t>6/9/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>v76; v84; v87; v93</t>
+          <t>v76; v84; v87; v93; v99</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>HXZ4HU: moved Excalibur (quest active)</t>
+          <t>HXZ4HU: moved Excalibur (quest active) | TP3TFA: moved Excalibur toward knights, quest active (t8)</t>
         </is>
       </c>
     </row>
@@ -2836,22 +2871,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>HXZ4HU; XF4V2C</t>
+          <t>HXZ4HU; XF4V2C; TP3TFA</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>6/12/2026; 6/13/2026</t>
+          <t>6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>v88; v91</t>
+          <t>v88; v91; v99</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Traitor Fate -&gt; opponents discard 2 (discard stuck pre-fix, fixed v88) | XF4V2C: opponents discard 2 (skip bug fixed v92)</t>
+          <t>Traitor Fate -&gt; opponents discard 2 (discard stuck pre-fix, fixed v88) | XF4V2C: opponents discard 2 (skip bug fixed v92) | TP3TFA: Percival Fate -&gt; opponents discard 2 (t12)</t>
         </is>
       </c>
     </row>
@@ -2873,22 +2908,22 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v93</t>
+          <t>v7x; v84; v87; v91; v93; v99</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>many placements + removals | XF4V2C: 3 placed (t17/t23/t30)</t>
+          <t>many placements + removals | XF4V2C: 3 placed (t17/t23/t30) | TP3TFA: 5 Despair placed (t2-t9)</t>
         </is>
       </c>
     </row>
@@ -2910,22 +2945,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>KLF2RQ; F2EXND</t>
+          <t>KLF2RQ; F2EXND; TP3TFA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>6/11/2026; 6/13/2026</t>
+          <t>6/11/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>v84; v92</t>
+          <t>v84; v92; v99</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>placed t28; replaced grail card t39 | F2EXND: placed t14; forced Grail loss t38</t>
+          <t>placed t28; replaced grail card t39 | F2EXND: placed t14; forced Grail loss t38 | TP3TFA: Desolation on Grail (t3)</t>
         </is>
       </c>
     </row>
@@ -2947,15 +2982,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>VJCEXL</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>46181</v>
+          <t>VJCEXL; TP3TFA</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>6/8/2026; 6/25/2026</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>v7x</t>
+          <t>v7x; v99</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>TP3TFA: Desolation quest-inactive -&gt; siege (t13)</t>
         </is>
       </c>
     </row>
@@ -3197,20 +3239,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>VJCEXL</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>46181</v>
+          <t>VJCEXL; TP3TFA</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>6/8/2026; 6/25/2026</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>v7x</t>
+          <t>v7x; v99</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>attached to Saxon War: +1 warrior, extra Fight 5 to win</t>
+          <t>attached to Saxon War: +1 warrior, extra Fight 5 to win | TP3TFA: attached to Saxon War, +1 warrior + extra Fight 5 (t11)</t>
         </is>
       </c>
     </row>
@@ -3378,22 +3422,22 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>tournament LOST 1x (6/8) and 2x (6/11-12) | HXZ4HU: tournament LOST | XF4V2C: Black Knight Tournament WON t17 (not via 4th this game) | F2EXND: 4th card forced combat -&gt; Tournament LOST t37</t>
+          <t>tournament LOST 1x (6/8) and 2x (6/11-12) | HXZ4HU: tournament LOST | XF4V2C: Black Knight Tournament WON t17 (not via 4th this game) | F2EXND: 4th card forced combat -&gt; Tournament LOST t37 | TP3TFA: Black Knight Tournament WON via fight cards (t23)</t>
         </is>
       </c>
     </row>
@@ -3452,22 +3496,22 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v93</t>
+          <t>v7x; v84; v87; v93; v99</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>both quests progressed/won in both games | HXZ4HU: Lancelot LOST t22; Dragon WON t35</t>
+          <t>both quests progressed/won in both games | HXZ4HU: Lancelot LOST t22; Dragon WON t35 | TP3TFA: Lancelot cards t8/t16; quest won t25</t>
         </is>
       </c>
     </row>
@@ -3489,22 +3533,22 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v93</t>
+          <t>v7x; v84; v87; v91; v93; v99</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>both the position-sink and quest-inactive siege variants | XF4V2C: Excalibur position sink t22/t31</t>
+          <t>both the position-sink and quest-inactive siege variants | XF4V2C: Excalibur position sink t22/t31 | TP3TFA: quest-inactive siege (t23)</t>
         </is>
       </c>
     </row>
@@ -3526,17 +3570,22 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>TP3TFA</t>
         </is>
       </c>
     </row>
@@ -3558,22 +3607,22 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>HXZ4HU: Dragon + siege | XF4V2C: BK/Lancelot/wars</t>
+          <t>HXZ4HU: Dragon + siege | XF4V2C: BK/Lancelot/wars | TP3TFA: Lancelot + Black Knight fights</t>
         </is>
       </c>
     </row>
@@ -3664,17 +3713,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TP3TFA</t>
         </is>
       </c>
     </row>
@@ -3770,22 +3824,22 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>many uses | XF4V2C: many | F2EXND: many</t>
+          <t>many uses | XF4V2C: many | F2EXND: many | TP3TFA: Percival t6, Arthur t7/t13, Galahad t8/t14</t>
         </is>
       </c>
     </row>
@@ -3807,22 +3861,22 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>4 divisions in KLF2RQ | HXZ4HU: Excalibur/Grail/Dragon divisions | XF4V2C: Pict War 4 cards; Convocation 2 | F2EXND: Saxon/Pict/Lancelot divisions</t>
+          <t>4 divisions in KLF2RQ | HXZ4HU: Excalibur/Grail/Dragon divisions | XF4V2C: Pict War 4 cards; Convocation 2 | F2EXND: Saxon/Pict/Lancelot divisions | TP3TFA: Excalibur 7 (t11), Black Knight 3 (t23), Lancelot 4 (t25)</t>
         </is>
       </c>
     </row>
@@ -3844,22 +3898,22 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>KLF2RQ; F2EXND</t>
+          <t>KLF2RQ; F2EXND; TP3TFA</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>6/11/2026; 6/13/2026</t>
+          <t>6/11/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>v84; v92</t>
+          <t>v84; v92; v99</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>host divided 3 cards | F2EXND: host divided 3 cards (setup)</t>
+          <t>host divided 3 cards | F2EXND: host divided 3 cards (setup) | TP3TFA: host divided 3 cards (setup)</t>
         </is>
       </c>
     </row>
@@ -3881,22 +3935,22 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>VJCEXL; HXZ4HU; XF4V2C; NEFE5L</t>
+          <t>VJCEXL; HXZ4HU; XF4V2C; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/12/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>v7x; v87; v91; v93</t>
+          <t>v7x; v87; v91; v93; v99</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>"Picky Safari forced a random distribution of 3 cards" | HXZ4HU: Chrome (setup); Arthur 7-card random (t35) | XF4V2C: Chrome forced random (setup)</t>
+          <t>"Picky Safari forced a random distribution of 3 cards" | HXZ4HU: Chrome (setup); Arthur 7-card random (t35) | XF4V2C: Chrome forced random (setup) | TP3TFA: Galahad 7-card forced random on Excalibur win (t11)</t>
         </is>
       </c>
     </row>
@@ -3918,17 +3972,22 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>TP3TFA</t>
         </is>
       </c>
     </row>
@@ -3950,17 +4009,22 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>VJCEXL; KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/8/2026; 6/11/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>v7x; v84; v87; v91; v92; v93</t>
+          <t>v7x; v84; v87; v91; v92; v93; v99</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>TP3TFA</t>
         </is>
       </c>
     </row>
@@ -4115,22 +4179,22 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L</t>
+          <t>KLF2RQ; HXZ4HU; XF4V2C; F2EXND; NEFE5L; TP3TFA</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>6/11-12/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026</t>
+          <t>6/11-12/2026; 6/12/2026; 6/13/2026; 6/13/2026; 6/13/2026; 6/25/2026</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>v84; v87; v91; v92; v93</t>
+          <t>v84; v87; v91; v92; v93; v99</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>148 passive kicks + 251 refocus heals; 0 stalls | HXZ4HU: heavy churn, recovered; 0 logic stalls | XF4V2C: heavy churn, recovered | F2EXND: long real-time gaps, recovered</t>
+          <t>148 passive kicks + 251 refocus heals; 0 stalls | HXZ4HU: heavy churn, recovered; 0 logic stalls | XF4V2C: heavy churn, recovered | F2EXND: long real-time gaps, recovered | TP3TFA: heartbeat-stale churn + refocus self-heals, 0 logic stalls</t>
         </is>
       </c>
     </row>

</xml_diff>